<commit_message>
결과 파일 업데이트 2026-08-14 10:04
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260814.xlsx
+++ b/results/andar_할인율모니터링_20260814.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H174"/>
+  <dimension ref="A1:H179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7,217</t>
+          <t>7,220</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>283</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>283</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>283</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4,932</t>
+          <t>4,933</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>9,943</t>
+          <t>9,944</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>209</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>3,408</t>
+          <t>3,409</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>3,408</t>
+          <t>3,409</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>679</t>
+          <t>680</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>266</t>
+          <t>267</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>3,135</t>
+          <t>3,137</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>3,135</t>
+          <t>3,137</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>125</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>661</t>
+          <t>662</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>1,058</t>
+          <t>1,060</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>247</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>96</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>202</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>1,340</t>
+          <t>1,341</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3809,7 +3809,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>1,340</t>
+          <t>1,341</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>1,340</t>
+          <t>1,341</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>1,520</t>
+          <t>1,521</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2,074</t>
+          <t>2,075</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>636</t>
+          <t>637</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -5153,7 +5153,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>73</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>547</t>
+          <t>548</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -6119,7 +6119,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>96</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -6781,12 +6781,12 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -6949,12 +6949,12 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>3,900</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>61%</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -7643,82 +7643,292 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12511&amp;cate_no=2111&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15151&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>ENTSO-03</t>
+          <t>EOTBG-22</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>안다르 이지무브 화이트</t>
+          <t>투포켓 로고 캔버스백</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>129,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>64,500</t>
+          <t>14,700</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>70%</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>496</t>
+          <t>21</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>EOTBG-05</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>메쉬 포켓 비치백</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>49,000</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>49,000</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=13843&amp;cate_no=2100&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>EOTBG-02</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>액티브 라이트 백팩</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>69,000</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>66,000</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>378</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=13842&amp;cate_no=2100&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>EOTBG-04</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>데님 포켓 숄더백</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>59,000</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>59,000</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=12778&amp;cate_no=2100&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>ENTBG-14</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>웨이브 패딩 파우치</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>32,000</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>32,000</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=12511&amp;cate_no=2111&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>ENTSO-03</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>안다르 이지무브 화이트</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>129,000</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>64,500</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>496</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
           <t>https://andar.co.kr/product/detail.html?product_no=12512&amp;cate_no=2111&amp;display_group=1</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr">
+      <c r="B179" t="inlineStr">
         <is>
           <t>ENTSO-03</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
+      <c r="C179" t="inlineStr">
         <is>
           <t>안다르 이지무브 베이지</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr">
+      <c r="D179" t="inlineStr">
         <is>
           <t>129,000</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr">
+      <c r="E179" t="inlineStr">
         <is>
           <t>64,500</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr">
+      <c r="F179" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr">
+      <c r="G179" t="inlineStr">
         <is>
           <t>414</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr">
+      <c r="H179" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>

</xml_diff>